<commit_message>
feat(xlsx): draw bubble, stock, treemap and sunburst charts from live cells
The Excel chart fixture generator now authors a bubble, an
open-high-low-close stock, a treemap and a sunburst chart in Excel, and the
fixture is regenerated. Bubble sizes resolve from live cells, and the
hidden _xlchart name behind a hierarchy's category range is replaced by the
range it stands for so the shared view can split its columns into levels
(outermost group first, leaf last). Editing a cell moves the chart.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/core/xlsx/__fixtures__/excel-chart-families.xlsx
+++ b/src/core/xlsx/__fixtures__/excel-chart-families.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Development\ooxml-core\.claude\worktrees\agent-a0c84f20aff81bc63\src\core\xlsx\__fixtures__\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Development\ooxml-core\.claude\worktrees\agent-a6c0f5fb5b9c1ff55\src\core\xlsx\__fixtures__\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D005397D-6B29-4264-B1B4-E44542CE6D6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5619D198-F96E-4D63-A3CA-5E0214F3246D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4180" yWindow="4180" windowWidth="28800" windowHeight="15370" xr2:uid="{63C83885-8987-490E-83EF-52A61F755AEF}"/>
+    <workbookView xWindow="1520" yWindow="1520" windowWidth="2200" windowHeight="1120" xr2:uid="{4FFBBD0A-EDEE-4A23-8B1C-D4B26ACC321C}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -21,10 +21,26 @@
     <definedName name="_xlchart.v1.10" hidden="1">Data!$B$2:$B$5</definedName>
     <definedName name="_xlchart.v1.11" hidden="1">Data!$C$1</definedName>
     <definedName name="_xlchart.v1.12" hidden="1">Data!$C$2:$C$5</definedName>
-    <definedName name="_xlchart.v1.13" hidden="1">Data!$H$1</definedName>
-    <definedName name="_xlchart.v1.14" hidden="1">Data!$H$2:$H$21</definedName>
+    <definedName name="_xlchart.v1.13" hidden="1">Data!$T$2:$U$6</definedName>
+    <definedName name="_xlchart.v1.14" hidden="1">Data!$V$1</definedName>
+    <definedName name="_xlchart.v1.15" hidden="1">Data!$V$2:$V$6</definedName>
+    <definedName name="_xlchart.v1.16" hidden="1">Data!$A$2:$A$5</definedName>
+    <definedName name="_xlchart.v1.17" hidden="1">Data!$B$1</definedName>
+    <definedName name="_xlchart.v1.18" hidden="1">Data!$B$2:$B$5</definedName>
+    <definedName name="_xlchart.v1.19" hidden="1">Data!$C$1</definedName>
     <definedName name="_xlchart.v1.2" hidden="1">Data!$B$2:$B$5</definedName>
+    <definedName name="_xlchart.v1.20" hidden="1">Data!$C$2:$C$5</definedName>
+    <definedName name="_xlchart.v1.21" hidden="1">Data!$H$1</definedName>
+    <definedName name="_xlchart.v1.22" hidden="1">Data!$H$2:$H$21</definedName>
+    <definedName name="_xlchart.v1.23" hidden="1">Data!$A$2:$A$5</definedName>
+    <definedName name="_xlchart.v1.24" hidden="1">Data!$B$1</definedName>
+    <definedName name="_xlchart.v1.25" hidden="1">Data!$B$2:$B$5</definedName>
+    <definedName name="_xlchart.v1.26" hidden="1">Data!$C$1</definedName>
+    <definedName name="_xlchart.v1.27" hidden="1">Data!$C$2:$C$5</definedName>
+    <definedName name="_xlchart.v1.28" hidden="1">Data!$T$2:$U$6</definedName>
+    <definedName name="_xlchart.v1.29" hidden="1">Data!$V$1</definedName>
     <definedName name="_xlchart.v1.3" hidden="1">Data!$C$1</definedName>
+    <definedName name="_xlchart.v1.30" hidden="1">Data!$V$2:$V$6</definedName>
     <definedName name="_xlchart.v1.4" hidden="1">Data!$C$2:$C$5</definedName>
     <definedName name="_xlchart.v1.5" hidden="1">Data!$E$2:$E$7</definedName>
     <definedName name="_xlchart.v1.6" hidden="1">Data!$F$1</definedName>
@@ -53,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="39">
   <si>
     <t>Quarter</t>
   </si>
@@ -101,6 +117,75 @@
   </si>
   <si>
     <t>Score</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>Size</t>
+  </si>
+  <si>
+    <t>Day</t>
+  </si>
+  <si>
+    <t>Open</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Close</t>
+  </si>
+  <si>
+    <t>Mon</t>
+  </si>
+  <si>
+    <t>Tue</t>
+  </si>
+  <si>
+    <t>Wed</t>
+  </si>
+  <si>
+    <t>Thu</t>
+  </si>
+  <si>
+    <t>Group</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>Weight</t>
+  </si>
+  <si>
+    <t>Fruit</t>
+  </si>
+  <si>
+    <t>Apple</t>
+  </si>
+  <si>
+    <t>Pear</t>
+  </si>
+  <si>
+    <t>Veg</t>
+  </si>
+  <si>
+    <t>Leek</t>
+  </si>
+  <si>
+    <t>Kale</t>
+  </si>
+  <si>
+    <t>Nuts</t>
+  </si>
+  <si>
+    <t>Almond</t>
   </si>
 </sst>
 </file>
@@ -298,7 +383,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-B6CE-4882-A507-23007DFAE67D}"/>
+              <c16:uniqueId val="{00000000-F417-4587-8D07-2C07082A1679}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -312,8 +397,8 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="1202705391"/>
-        <c:axId val="1086017391"/>
+        <c:axId val="731296831"/>
+        <c:axId val="733517615"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -400,7 +485,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-B6CE-4882-A507-23007DFAE67D}"/>
+              <c16:uniqueId val="{00000001-F417-4587-8D07-2C07082A1679}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -414,11 +499,11 @@
         </c:dLbls>
         <c:marker val="1"/>
         <c:smooth val="0"/>
-        <c:axId val="1206901551"/>
-        <c:axId val="1086014511"/>
+        <c:axId val="731295439"/>
+        <c:axId val="733522895"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1202705391"/>
+        <c:axId val="731296831"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -461,7 +546,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1086017391"/>
+        <c:crossAx val="733517615"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -469,7 +554,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1086017391"/>
+        <c:axId val="733517615"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -520,12 +605,12 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1202705391"/>
+        <c:crossAx val="731296831"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="1086014511"/>
+        <c:axId val="733522895"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -562,12 +647,12 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1206901551"/>
+        <c:crossAx val="731295439"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="1206901551"/>
+        <c:axId val="731295439"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -577,12 +662,977 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1086014511"/>
+        <c:crossAx val="733522895"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Bubbles</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:bubbleChart>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Points</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1">
+                <a:alpha val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln w="25400">
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Data!$J$2:$J$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Data!$K$2:$K$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:bubbleSize>
+            <c:numRef>
+              <c:f>Data!$L$2:$L$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:bubbleSize>
+          <c:bubble3D val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-C027-4088-8B08-E016A95183FF}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:bubbleScale val="100"/>
+        <c:showNegBubbles val="0"/>
+        <c:axId val="295511568"/>
+        <c:axId val="733521935"/>
+      </c:bubbleChart>
+      <c:valAx>
+        <c:axId val="295511568"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="733521935"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="733521935"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="295511568"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Prices</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:stockChart>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Data!$O$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Open</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Data!$N$2:$N$5</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Mon</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Tue</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Wed</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Thu</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Data!$O$2:$O$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>11</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-F600-4161-AFBA-A35CF34D5402}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Data!$P$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>High</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Data!$N$2:$N$5</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Mon</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Tue</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Wed</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Thu</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Data!$P$2:$P$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>14</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-F600-4161-AFBA-A35CF34D5402}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Data!$Q$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Low</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Data!$N$2:$N$5</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Mon</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Tue</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Wed</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Thu</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Data!$Q$2:$Q$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>9</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-F600-4161-AFBA-A35CF34D5402}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Data!$R$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Close</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Data!$N$2:$N$5</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Mon</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Tue</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Wed</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Thu</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Data!$R$2:$R$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>13</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-F600-4161-AFBA-A35CF34D5402}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:hiLowLines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="75000"/>
+                  <a:lumOff val="25000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:hiLowLines>
+        <c:upDownBars>
+          <c:gapWidth val="219"/>
+          <c:upBars>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="15000"/>
+                    <a:lumOff val="85000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:upBars>
+          <c:downBars>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="dk1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:downBars>
+        </c:upDownBars>
+        <c:axId val="295506928"/>
+        <c:axId val="733524335"/>
+      </c:stockChart>
+      <c:catAx>
+        <c:axId val="295506928"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="733524335"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="733524335"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="295506928"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
       <c:spPr>
         <a:noFill/>
         <a:ln>
@@ -688,7 +1738,7 @@
     </cx:title>
     <cx:plotArea>
       <cx:plotAreaRegion>
-        <cx:series layoutId="waterfall" uniqueId="{00000002-7633-4370-8AB4-9599B63ABCEC}">
+        <cx:series layoutId="waterfall" uniqueId="{00000002-B75B-4498-9D58-5DB68578D3EB}">
           <cx:tx>
             <cx:txData>
               <cx:f>_xlchart.v1.6</cx:f>
@@ -725,7 +1775,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.14</cx:f>
+        <cx:f>_xlchart.v1.22</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -739,10 +1789,10 @@
     </cx:title>
     <cx:plotArea>
       <cx:plotAreaRegion>
-        <cx:series layoutId="clusteredColumn" uniqueId="{00000002-F734-47EB-B6B3-38E9BC491DB8}">
+        <cx:series layoutId="clusteredColumn" uniqueId="{00000002-DA57-47C5-B5EB-411E5EC074B2}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.13</cx:f>
+              <cx:f>_xlchart.v1.21</cx:f>
               <cx:v>Score</cx:v>
             </cx:txData>
           </cx:tx>
@@ -761,6 +1811,82 @@
         <cx:majorGridlines/>
         <cx:tickLabels/>
       </cx:axis>
+    </cx:plotArea>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
+<file path=xl/charts/chartEx3.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:strDim type="cat">
+        <cx:f>_xlchart.v1.13</cx:f>
+      </cx:strDim>
+      <cx:numDim type="size">
+        <cx:f>_xlchart.v1.15</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0">
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Produce treemap</cx:v>
+        </cx:txData>
+      </cx:tx>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="treemap" uniqueId="{00000002-60C6-475A-A842-57D6B71BB076}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.14</cx:f>
+              <cx:v>Weight</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="0"/>
+          <cx:layoutPr/>
+        </cx:series>
+      </cx:plotAreaRegion>
+    </cx:plotArea>
+    <cx:legend pos="t" align="ctr" overlay="0"/>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
+<file path=xl/charts/chartEx4.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:strDim type="cat">
+        <cx:f>_xlchart.v1.28</cx:f>
+      </cx:strDim>
+      <cx:numDim type="size">
+        <cx:f>_xlchart.v1.30</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0">
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Produce sunburst</cx:v>
+        </cx:txData>
+      </cx:tx>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="sunburst" uniqueId="{00000002-10B3-453A-9ED3-4722716C7E29}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.29</cx:f>
+              <cx:v>Weight</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="0"/>
+        </cx:series>
+      </cx:plotAreaRegion>
     </cx:plotArea>
   </cx:chart>
 </cx:chartSpace>
@@ -886,6 +2012,166 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors6.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors7.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
@@ -2010,6 +3296,2076 @@
       <a:solidFill>
         <a:schemeClr val="phClr"/>
       </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat">
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="269">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr">
+          <a:alpha val="75000"/>
+        </a:schemeClr>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr">
+          <a:alpha val="75000"/>
+        </a:schemeClr>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:alpha val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style6.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="410">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1">
+          <a:lumMod val="65000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="bg1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat">
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style7.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="381">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
     </cs:spPr>
   </cs:dataPoint>
   <cs:dataPoint3D>
@@ -2425,7 +5781,7 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{39EA0563-34E7-4E3E-E9CE-44A627914593}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{21D8C238-0102-0B18-3E1E-AFDE3E86E408}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2463,7 +5819,7 @@
             <xdr:cNvPr id="3" name="Chart 2">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{43257927-01A7-291B-1D94-AC1DE78475F3}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B1315B41-CD3A-0503-9465-1EB92254937C}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2541,7 +5897,7 @@
             <xdr:cNvPr id="4" name="Chart 3">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{87253B85-1ED3-B6D9-457A-831651FF5B0D}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5E93D77A-8337-1204-922B-BDC0C4AA7D90}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2569,6 +5925,234 @@
           <xdr:spPr>
             <a:xfrm>
               <a:off x="9906000" y="2540000"/>
+              <a:ext cx="4572000" cy="2794000"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100"/>
+                <a:t>This chart isn't available in your version of Excel.
+Editing this shape or saving this workbook into a different file format will permanently break the chart.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>254000</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>558800</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A9EA1319-1181-56FF-7C47-FBA4C98168DD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>203200</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>508000</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Chart 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2810678E-6456-A446-620B-28AC931CC7A5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>152400</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>457200</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="7" name="Chart 6">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{58BA704F-A969-7397-D0C5-2F658C37D317}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
+              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="9906000" y="5588000"/>
+              <a:ext cx="4572000" cy="2794000"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100"/>
+                <a:t>This chart isn't available in your version of Excel.
+Editing this shape or saving this workbook into a different file format will permanently break the chart.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>101600</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>406400</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="8" name="Chart 7">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A7BC070A-5321-8DBC-6335-158AA64A7778}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
+              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="14732000" y="5588000"/>
               <a:ext cx="4572000" cy="2794000"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -2918,11 +6502,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D594A7F3-8774-4740-8351-1E4E06451589}">
-  <dimension ref="A1:H21"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B974F96D-3B35-4B07-A253-3347617234C6}">
+  <dimension ref="A1:V21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2941,8 +6525,41 @@
       <c r="H1" t="s">
         <v>15</v>
       </c>
+      <c r="J1" t="s">
+        <v>16</v>
+      </c>
+      <c r="K1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L1" t="s">
+        <v>18</v>
+      </c>
+      <c r="N1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O1" t="s">
+        <v>20</v>
+      </c>
+      <c r="P1" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>22</v>
+      </c>
+      <c r="R1" t="s">
+        <v>23</v>
+      </c>
+      <c r="T1" t="s">
+        <v>28</v>
+      </c>
+      <c r="U1" t="s">
+        <v>29</v>
+      </c>
+      <c r="V1" t="s">
+        <v>30</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2961,8 +6578,41 @@
       <c r="H2">
         <v>3</v>
       </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>3</v>
+      </c>
+      <c r="L2">
+        <v>5</v>
+      </c>
+      <c r="N2" t="s">
+        <v>24</v>
+      </c>
+      <c r="O2">
+        <v>10</v>
+      </c>
+      <c r="P2">
+        <v>14</v>
+      </c>
+      <c r="Q2">
+        <v>9</v>
+      </c>
+      <c r="R2">
+        <v>12</v>
+      </c>
+      <c r="T2" t="s">
+        <v>31</v>
+      </c>
+      <c r="U2" t="s">
+        <v>32</v>
+      </c>
+      <c r="V2">
+        <v>30</v>
+      </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -2981,8 +6631,41 @@
       <c r="H3">
         <v>5</v>
       </c>
+      <c r="J3">
+        <v>2</v>
+      </c>
+      <c r="K3">
+        <v>5</v>
+      </c>
+      <c r="L3">
+        <v>10</v>
+      </c>
+      <c r="N3" t="s">
+        <v>25</v>
+      </c>
+      <c r="O3">
+        <v>11</v>
+      </c>
+      <c r="P3">
+        <v>15</v>
+      </c>
+      <c r="Q3">
+        <v>10</v>
+      </c>
+      <c r="R3">
+        <v>13</v>
+      </c>
+      <c r="T3" t="s">
+        <v>31</v>
+      </c>
+      <c r="U3" t="s">
+        <v>33</v>
+      </c>
+      <c r="V3">
+        <v>20</v>
+      </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -3001,8 +6684,41 @@
       <c r="H4">
         <v>7</v>
       </c>
+      <c r="J4">
+        <v>3</v>
+      </c>
+      <c r="K4">
+        <v>4</v>
+      </c>
+      <c r="L4">
+        <v>3</v>
+      </c>
+      <c r="N4" t="s">
+        <v>26</v>
+      </c>
+      <c r="O4">
+        <v>12</v>
+      </c>
+      <c r="P4">
+        <v>15</v>
+      </c>
+      <c r="Q4">
+        <v>10</v>
+      </c>
+      <c r="R4">
+        <v>11</v>
+      </c>
+      <c r="T4" t="s">
+        <v>34</v>
+      </c>
+      <c r="U4" t="s">
+        <v>35</v>
+      </c>
+      <c r="V4">
+        <v>10</v>
+      </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -3021,8 +6737,41 @@
       <c r="H5">
         <v>8</v>
       </c>
+      <c r="J5">
+        <v>4</v>
+      </c>
+      <c r="K5">
+        <v>8</v>
+      </c>
+      <c r="L5">
+        <v>8</v>
+      </c>
+      <c r="N5" t="s">
+        <v>27</v>
+      </c>
+      <c r="O5">
+        <v>11</v>
+      </c>
+      <c r="P5">
+        <v>14</v>
+      </c>
+      <c r="Q5">
+        <v>9</v>
+      </c>
+      <c r="R5">
+        <v>13</v>
+      </c>
+      <c r="T5" t="s">
+        <v>34</v>
+      </c>
+      <c r="U5" t="s">
+        <v>36</v>
+      </c>
+      <c r="V5">
+        <v>5</v>
+      </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
       <c r="E6" t="s">
         <v>13</v>
       </c>
@@ -3032,8 +6781,17 @@
       <c r="H6">
         <v>8</v>
       </c>
+      <c r="T6" t="s">
+        <v>37</v>
+      </c>
+      <c r="U6" t="s">
+        <v>38</v>
+      </c>
+      <c r="V6">
+        <v>8</v>
+      </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
       <c r="E7" t="s">
         <v>14</v>
       </c>
@@ -3044,47 +6802,47 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
       <c r="H8">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
       <c r="H9">
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
       <c r="H10">
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
       <c r="H11">
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
       <c r="H12">
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
       <c r="H13">
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.35">
       <c r="H14">
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.35">
       <c r="H15">
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.35">
       <c r="H16">
         <v>18</v>
       </c>

</xml_diff>